<commit_message>
Refined documentation and code structure for clarity and accuracy. Updated README and alpha build documentation to reflect changes in routing and ticketing processes. Adjusted API response models to return tickets for unclear sections and improved draft function to include passage IDs. Enhanced evaluation criteria to align with new routing logic.
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CFBDB3E-912B-4E85-B01E-9EB55BCD2544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E37BE4-D438-49AD-9546-242C8F5E3ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="182">
   <si>
     <t>Sprint tasks</t>
   </si>
@@ -137,7 +137,7 @@
     <t>Ask the chat model for a section id or “unclear”. The graph accepts only appointments, referrals_waiting, records_results, or unclear.</t>
   </si>
   <si>
-    <t>When the section is clear, skip the clarifying question and retrieve only that section.</t>
+    <t>When the section is clear, retrieve only that section.</t>
   </si>
   <si>
     <t>Route “How can I change my hospital appointment?” to Appointments, and do not answer it from another section.</t>
@@ -149,19 +149,19 @@
     <t>4</t>
   </si>
   <si>
-    <t>Clarify and escalate</t>
-  </si>
-  <si>
-    <t>Fix the clarifying sentence. It names Appointments, Referrals &amp; Waiting, and Records &amp; Results, and it states no policy.</t>
+    <t>Escalate and clinical boundary</t>
+  </si>
+  <si>
+    <t>When the section is not clear, open a ticket with no section and state no policy.</t>
   </si>
   <si>
     <t>When the section is unclear, send that one question. The first reply contains no citation and no ticket. No edge leads back to a second question.</t>
   </si>
   <si>
-    <t>On the second turn, accept only one of the three section ids, or unclear. A reply that names a section continues. A reply that does not opens a ticket with no section.</t>
-  </si>
-  <si>
-    <t>Show the one clarifying question on “I’ve been referred but haven’t heard anything about my appointment.”</t>
+    <t>An unclear label opens a ticket with no section. The person is not asked to choose a section.</t>
+  </si>
+  <si>
+    <t>Show a ticket with no section for a question that could belong to more than one section.</t>
   </si>
   <si>
     <t>When the right section’s pages do not support the answer, open a ticket for that section. The reply says the guidance is insufficient. A missing wait is not invented.</t>
@@ -206,7 +206,7 @@
     <t>Cover the target shape: clear routing (6), ambiguous routing (4), cross-domain (3), answerable (3), unsupported (2), escalation (2), plus clinical-boundary questions.</t>
   </si>
   <si>
-    <t>Give each row a question, a section label, a category, an expected ending, a scripted reply on two-turn cases, and a should-answer flag.</t>
+    <t>Give each row a question, a section label, a category, an expected ending, and a should-answer flag.</t>
   </si>
   <si>
     <t>Freeze the set. Leave the questions fixed while tuning. Do not edit a question after a model answer has been seen.</t>
@@ -233,13 +233,13 @@
     <t>UAT</t>
   </si>
   <si>
-    <t>A1. Send each golden item and compare the section id. A clear question is not asked to clarify.</t>
+    <t>A1. Send each golden item and compare the section id.</t>
   </si>
   <si>
     <t>A2 and A3. An in-policy question returns evidence, and the source URL belongs to the routed section.</t>
   </si>
   <si>
-    <t>A5 and A6. The first body is one clarifying question with an empty ticket. If the reply names nothing, the second body is a ticket with an empty section.</t>
+    <t>A5 and A6. An unclear section is a ticket with no section and no policy.</t>
   </si>
   <si>
     <t>A4 and A10. A gap in the right section is a ticket for that section. The body claims no missing rule, and it says the guidance is insufficient.</t>
@@ -341,7 +341,7 @@
     <t>“How can I change my hospital appointment?” is routed to Appointments and is not answered from another section.</t>
   </si>
   <si>
-    <t>A1. A clear question is routed immediately and is not asked to clarify.</t>
+    <t>A1. A clear question is routed and answered.</t>
   </si>
   <si>
     <t>The model suggests a section id or “unclear”. The graph accepts only appointments, referrals_waiting, records_results, or unclear.</t>
@@ -350,7 +350,7 @@
     <t>3. Routing</t>
   </si>
   <si>
-    <t>The one clarifying question, the second turn, both ticket reasons, and the clinical signpost.</t>
+    <t>Both ticket reasons and the clinical signpost.</t>
   </si>
   <si>
     <t>“I’ve been referred but haven’t heard anything about my appointment” asks once. An unclear reply, and a missing wait, each open a ticket. “What does this test result mean for me?” signposts and states no clinical advice.</t>
@@ -359,10 +359,10 @@
     <t>A4, A5, A6, A8, A10.</t>
   </si>
   <si>
-    <t>The clarifying sentence and the signpost are fixed wording, written with the code. One question is the limit. Ticket reasons: the section was still unclear, or the pages do not support an answer. A stored chat session waits until a second interface exists.</t>
-  </si>
-  <si>
-    <t>4. Clarify and escalate</t>
+    <t>The signpost is fixed wording, written with the code. One request carries one question. Ticket reasons: the section was not clear, or the pages do not support an answer.</t>
+  </si>
+  <si>
+    <t>4. Escalate and clinical boundary</t>
   </si>
   <si>
     <t>Retrieval filtered by section_id, checked on all six directed pairs.</t>
@@ -395,7 +395,7 @@
     <t>6. Evaluation</t>
   </si>
   <si>
-    <t>The discovery script, run against Docker: route labels, two-turn clarifying cases, clinical-boundary cases, the leak test, and one RAGAS run.</t>
+    <t>The discovery script, run against Docker: route labels, unclear-section tickets, clinical-boundary cases, the leak test, and one RAGAS run.</t>
   </si>
   <si>
     <t>Every acceptance criterion is shown, including one RAGAS run.</t>
@@ -449,7 +449,7 @@
     <t>Correct domain</t>
   </si>
   <si>
-    <t>A question about one section is not answered from another. On the golden set, the route matches the label written in advance. A question whose section is already clear is routed immediately, and no clarifying question is asked.</t>
+    <t>A question about one section is not answered from another. On the golden set, the route matches the label written in advance. A question whose section is already clear is routed and answered.</t>
   </si>
   <si>
     <t>7. Docker UAT</t>
@@ -500,7 +500,7 @@
     <t>Ambiguity</t>
   </si>
   <si>
-    <t>When the question could reasonably belong to more than one section, Deskline may ask one clarifying question. The question names the three sections and states no policy. The first reply contains no citation and no ticket.</t>
+    <t>When the question could reasonably belong to more than one section, Deskline opens a ticket with no section. The reply states no policy and contains no citation.</t>
   </si>
   <si>
     <t>pytest checks the first body for a question and an empty ticket.</t>
@@ -512,7 +512,7 @@
     <t>Still unclear</t>
   </si>
   <si>
-    <t>When the reply does not establish an answerable section, Deskline escalates. The ticket has no section and no policy statement. A second clarifying question is not asked.</t>
+    <t>When the question belongs to none of the three sections, Deskline opens a ticket with no section and no policy statement. The person is not asked to choose a section.</t>
   </si>
   <si>
     <t>pytest checks the second body for a ticket and an empty section.</t>
@@ -576,9 +576,6 @@
   </si>
   <si>
     <t>The eval runner, started by hand, writes an eval-run row. The first run is kept even if it is below 0.8.</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -722,12 +719,12 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1154,7 +1151,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>84</v>
       </c>
       <c r="B1" s="13"/>
@@ -1167,7 +1164,7 @@
       <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>85</v>
       </c>
       <c r="B2" s="13"/>
@@ -1289,7 +1286,7 @@
         <v>103</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>104</v>
@@ -1491,7 +1488,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -1501,7 +1498,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -1829,7 +1826,7 @@
         <v>31</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>182</v>
+        <v>11</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="8" t="s">
@@ -1847,7 +1844,7 @@
         <v>34</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="8" t="s">
@@ -1865,7 +1862,7 @@
         <v>35</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="8" t="s">
@@ -1883,7 +1880,7 @@
         <v>36</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="8" t="s">
@@ -2572,7 +2569,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>130</v>
       </c>
       <c r="B1" s="13"/>
@@ -2582,7 +2579,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>131</v>
       </c>
       <c r="B2" s="13"/>

</xml_diff>

<commit_message>
removed the fewshot examples
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E37BE4-D438-49AD-9546-242C8F5E3ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1876E05-FB8B-489D-8B8E-EBE682C8610D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -719,12 +719,12 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1151,7 +1151,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>84</v>
       </c>
       <c r="B1" s="13"/>
@@ -1164,7 +1164,7 @@
       <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>85</v>
       </c>
       <c r="B2" s="13"/>
@@ -1488,7 +1488,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -1498,7 +1498,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -1898,7 +1898,7 @@
         <v>37</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="8" t="s">
@@ -2569,7 +2569,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>130</v>
       </c>
       <c r="B1" s="13"/>
@@ -2579,7 +2579,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>131</v>
       </c>
       <c r="B2" s="13"/>

</xml_diff>

<commit_message>
sprint 4 is done
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1876E05-FB8B-489D-8B8E-EBE682C8610D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C3C1A8-A8E6-430C-AFAD-99145597C6B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprints" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="183">
   <si>
     <t>Sprint tasks</t>
   </si>
@@ -576,6 +576,9 @@
   </si>
   <si>
     <t>The eval runner, started by hand, writes an eval-run row. The first run is kept even if it is below 0.8.</t>
+  </si>
+  <si>
+    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -1315,7 +1318,7 @@
         <v>108</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>109</v>
@@ -1344,7 +1347,7 @@
         <v>113</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>24</v>
+        <v>182</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>114</v>
@@ -1916,7 +1919,7 @@
         <v>40</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="8" t="s">
@@ -1934,7 +1937,7 @@
         <v>41</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="8" t="s">
@@ -1952,7 +1955,7 @@
         <v>42</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="8" t="s">
@@ -1970,7 +1973,7 @@
         <v>43</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="8" t="s">
@@ -1988,7 +1991,7 @@
         <v>44</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="8" t="s">
@@ -2006,7 +2009,7 @@
         <v>45</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="8" t="s">
@@ -2024,7 +2027,7 @@
         <v>46</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E31" s="7"/>
       <c r="F31" s="8" t="s">
@@ -2042,7 +2045,7 @@
         <v>47</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="8" t="s">

</xml_diff>

<commit_message>
Implement section validation and refine passage retrieval in search functionality. Added checks for allowed section IDs and ensured only relevant passages are returned, raising errors for unknown sections or foreign passages. api is containerised , the golden set is created
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C3C1A8-A8E6-430C-AFAD-99145597C6B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ECEBA2-CAB6-465C-9D48-14C92FF98548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprints" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Acceptance!$A$3:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sprints!$A$3:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Tasks!$A$3:$F$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Tasks!$A$3:$F$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">Acceptance!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Sprints!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">Tasks!$1:$3</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="178">
   <si>
     <t>Sprint tasks</t>
   </si>
@@ -182,18 +182,6 @@
     <t>Isolation</t>
   </si>
   <si>
-    <t>Filter retrieval by section_id. Load passages only for the chosen section, and only from documents in the approved corpus.</t>
-  </si>
-  <si>
-    <t>Run the leak test on all six directed pairs. An Appointments query returns no Referrals &amp; Waiting or Records &amp; Results passage, and the same for the other pairs.</t>
-  </si>
-  <si>
-    <t>Call retrieval directly in the leak test. Do not ask the chat model whether the answer sounds like the right section.</t>
-  </si>
-  <si>
-    <t>Add tests/leakage/ for A7, and tests/retrieval/ for the citation and approved-corpus checks (A2, A3, A9).</t>
-  </si>
-  <si>
     <t>6</t>
   </si>
   <si>
@@ -374,9 +362,6 @@
     <t>A7. A9 is the approved-corpus check beside it.</t>
   </si>
   <si>
-    <t>The leak test calls retrieval directly. It does not ask the chat model whether the answer sounds like the right section. The six pairs are only meaningful because the corpus shares vocabulary.</t>
-  </si>
-  <si>
     <t>5. Isolation</t>
   </si>
   <si>
@@ -578,7 +563,7 @@
     <t>The eval runner, started by hand, writes an eval-run row. The first run is kept even if it is below 0.8.</t>
   </si>
   <si>
-    <t>In progress</t>
+    <t>Two checks run on every search. An id that is not one of the three never reaches the database. After the database answers, every passage must still carry that same section_id. A passage from another section raises, so it is not handed to the draft.</t>
   </si>
 </sst>
 </file>
@@ -722,12 +707,12 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1154,8 +1139,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>84</v>
+      <c r="A1" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1167,8 +1152,8 @@
       <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>85</v>
+      <c r="A2" s="14" t="s">
+        <v>81</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -1190,16 +1175,16 @@
         <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>5</v>
@@ -1219,22 +1204,22 @@
         <v>12</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
@@ -1248,22 +1233,22 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
@@ -1277,22 +1262,22 @@
         <v>12</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
@@ -1306,22 +1291,22 @@
         <v>12</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
@@ -1335,109 +1320,109 @@
         <v>12</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>182</v>
+        <v>11</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>114</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>24</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>24</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>24</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1479,7 +1464,7 @@
     <tabColor rgb="FF1F6F6A"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1491,7 +1476,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -1501,7 +1486,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -2060,10 +2045,10 @@
         <v>49</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>50</v>
+        <v>177</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="8" t="s">
@@ -2072,13 +2057,13 @@
     </row>
     <row r="34" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>24</v>
@@ -2090,13 +2075,13 @@
     </row>
     <row r="35" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>24</v>
@@ -2108,13 +2093,13 @@
     </row>
     <row r="36" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>24</v>
@@ -2126,13 +2111,13 @@
     </row>
     <row r="37" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>24</v>
@@ -2144,13 +2129,13 @@
     </row>
     <row r="38" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>24</v>
@@ -2162,13 +2147,13 @@
     </row>
     <row r="39" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>24</v>
@@ -2180,13 +2165,13 @@
     </row>
     <row r="40" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>24</v>
@@ -2197,65 +2182,65 @@
       </c>
     </row>
     <row r="41" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>55</v>
+      <c r="A41" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E41" s="7"/>
-      <c r="F41" s="8" t="s">
-        <v>12</v>
+      <c r="F41" s="9" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>55</v>
+      <c r="A42" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E42" s="7"/>
-      <c r="F42" s="8" t="s">
-        <v>12</v>
+      <c r="F42" s="9" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>55</v>
+      <c r="A43" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E43" s="7"/>
-      <c r="F43" s="8" t="s">
-        <v>12</v>
+      <c r="F43" s="9" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>65</v>
@@ -2265,159 +2250,159 @@
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E46" s="7"/>
       <c r="F46" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>64</v>
+      <c r="A50" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D50" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E50" s="7"/>
-      <c r="F50" s="9" t="s">
-        <v>66</v>
+      <c r="F50" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>64</v>
+      <c r="A51" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E51" s="7"/>
-      <c r="F51" s="9" t="s">
-        <v>66</v>
+      <c r="F51" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>64</v>
+      <c r="A52" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D52" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E52" s="7"/>
-      <c r="F52" s="9" t="s">
-        <v>66</v>
+      <c r="F52" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C53" s="7" t="s">
         <v>77</v>
@@ -2427,110 +2412,56 @@
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E54" s="7"/>
       <c r="F54" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E56" s="7"/>
-      <c r="F56" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E57" s="7"/>
-      <c r="F57" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E58" s="7"/>
-      <c r="F58" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F58" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F58">
-      <sortCondition ref="A4:A100"/>
+  <autoFilter ref="A3:F55" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F55">
+      <sortCondition ref="A4:A97"/>
     </sortState>
   </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D4:D58">
+  <conditionalFormatting sqref="D4:D55">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>D4="Not started"</formula>
     </cfRule>
@@ -2545,7 +2476,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Choose a status from the list" promptTitle="Status" prompt="Not started, In progress, Done, or Blocked" sqref="D4:D58" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Choose a status from the list" promptTitle="Status" prompt="Not started, In progress, Done, or Blocked" sqref="D4:D55" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Not started,In progress,Done,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2572,8 +2503,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>130</v>
+      <c r="A1" s="12" t="s">
+        <v>125</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -2582,8 +2513,8 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>131</v>
+      <c r="A2" s="14" t="s">
+        <v>126</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -2593,242 +2524,242 @@
     </row>
     <row r="3" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>140</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 7 is complete as a record. Calls 1, 2, and 5 passed. Calls 3 and 4 missed, and the plan starts Azure only after every acceptance rule has passed. For this proof of concept that record stays as it is, and the next thing to learn is sprint 8: the same shape on Azure, without the pages.
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C52AD8-7141-48F8-A3F4-1660B906B9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA91352-7501-4977-AF63-2A1F48D72781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -707,12 +707,12 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1139,7 +1139,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>80</v>
       </c>
       <c r="B1" s="13"/>
@@ -1152,7 +1152,7 @@
       <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>81</v>
       </c>
       <c r="B2" s="13"/>
@@ -1390,7 +1390,7 @@
         <v>118</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>119</v>
@@ -1476,7 +1476,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -1486,7 +1486,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -2192,7 +2192,7 @@
         <v>61</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="9" t="s">
@@ -2210,7 +2210,7 @@
         <v>63</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="9" t="s">
@@ -2228,7 +2228,7 @@
         <v>64</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="9" t="s">
@@ -2246,7 +2246,7 @@
         <v>65</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="9" t="s">
@@ -2264,7 +2264,7 @@
         <v>66</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="9" t="s">
@@ -2282,7 +2282,7 @@
         <v>67</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E46" s="7"/>
       <c r="F46" s="9" t="s">
@@ -2300,7 +2300,7 @@
         <v>68</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="9" t="s">
@@ -2318,7 +2318,7 @@
         <v>69</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="9" t="s">
@@ -2336,7 +2336,7 @@
         <v>70</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="9" t="s">
@@ -2503,7 +2503,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>125</v>
       </c>
       <c r="B1" s="13"/>
@@ -2513,7 +2513,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>126</v>
       </c>
       <c r="B2" s="13"/>

</xml_diff>

<commit_message>
notes about the rollout phase
</commit_message>
<xml_diff>
--- a/docs/sprints.xlsx
+++ b/docs/sprints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramy\my projects\Deskline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA91352-7501-4977-AF63-2A1F48D72781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83C42EEB-577F-4C54-81ED-25CF44BD7701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprints" sheetId="1" r:id="rId1"/>
@@ -1419,7 +1419,7 @@
         <v>123</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>124</v>

</xml_diff>